<commit_message>
Re-extrakce poškozených extraligových tabulek z originálních PDF (80→0 buněk)
Zdroj: sources/CZE1/CZ-YYYY-YY.pdf (+ sources/CZE2_3_nizsi/) — kompletní a přesný.

fill_from_pdf.py doplnil/opravil 9 sezón:
- 1980/81, 1981/82: celé tabulky (GA chyběla, řádek posunutý; 4 sl. V/VP/PP/P, bez remíz) → W=V+VP, D=0, L=PP+P, GF/GA/PTS
- 2000/01, 2001/02: doplněny GA+PTS, opraveno W/D/L (3-bodový systém od 2000/01)
- 1991/92–1995/96: rozdělené ligy/nadstavba — opraven 5-sloupcový V/VP/R/PP/P cram (W/D/L/GF/GA/PTS)

Každý řádek ověřen: suma GF=suma GA, V+R+P=GP, křížově proti xlsx. Žádná data se nevymýšlela.

validate_almanach.py: PTS=2V+R kontrola jen pro <2000 (3-body od 2000/01); §4 reziduální anomálie (1988/89 přenos bodů = korektní; 3× ±1 v ZČ k ověření).
Přidány zdrojové PDF do sources/ (self-contained, re-runnable). README + MASTER_REPORT aktualizovány.
</commit_message>
<xml_diff>
--- a/data/S1980_81_FINAL.xlsx
+++ b/data/S1980_81_FINAL.xlsx
@@ -29,7 +29,7 @@
     <sheet name="TODO" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'TODO'!$A$1:$F$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'TODO'!$A$1:$F$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -718,29 +718,27 @@
         <v>44</v>
       </c>
       <c r="G4" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="H4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J4" t="n">
-        <v>9</v>
+        <v>211</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L4" t="n">
+        <v>148</v>
       </c>
       <c r="M4" t="n">
-        <v>148</v>
+        <v>68</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -806,29 +804,27 @@
         <v>44</v>
       </c>
       <c r="G5" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>193</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L5" t="n">
+        <v>119</v>
       </c>
       <c r="M5" t="n">
-        <v>119</v>
+        <v>66</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -894,29 +890,27 @@
         <v>44</v>
       </c>
       <c r="G6" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J6" t="n">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L6" t="n">
+        <v>124</v>
       </c>
       <c r="M6" t="n">
-        <v>124</v>
+        <v>58</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -982,29 +976,27 @@
         <v>44</v>
       </c>
       <c r="G7" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="J7" t="n">
-        <v>15</v>
+        <v>177</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L7" t="n">
+        <v>131</v>
       </c>
       <c r="M7" t="n">
-        <v>131</v>
+        <v>52</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -1070,29 +1062,27 @@
         <v>44</v>
       </c>
       <c r="G8" t="n">
+        <v>25</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
         <v>19</v>
       </c>
-      <c r="H8" t="n">
-        <v>6</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
       <c r="J8" t="n">
-        <v>18</v>
+        <v>170</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L8" t="n">
+        <v>173</v>
       </c>
       <c r="M8" t="n">
-        <v>173</v>
+        <v>50</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -1158,29 +1148,27 @@
         <v>44</v>
       </c>
       <c r="G9" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="J9" t="n">
-        <v>23</v>
+        <v>158</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L9" t="n">
+        <v>181</v>
       </c>
       <c r="M9" t="n">
-        <v>181</v>
+        <v>40</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1246,29 +1234,27 @@
         <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="J10" t="n">
-        <v>22</v>
+        <v>169</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L10" t="n">
+        <v>190</v>
       </c>
       <c r="M10" t="n">
-        <v>190</v>
+        <v>38</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1334,29 +1320,27 @@
         <v>44</v>
       </c>
       <c r="G11" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="J11" t="n">
-        <v>23</v>
+        <v>155</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L11" t="n">
+        <v>178</v>
       </c>
       <c r="M11" t="n">
-        <v>178</v>
+        <v>36</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1428,23 +1412,21 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="J12" t="n">
-        <v>23</v>
+        <v>176</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L12" t="n">
+        <v>199</v>
       </c>
       <c r="M12" t="n">
-        <v>199</v>
+        <v>34</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1521,23 +1503,21 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="J13" t="n">
-        <v>28</v>
+        <v>125</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L13" t="n">
+        <v>161</v>
       </c>
       <c r="M13" t="n">
-        <v>161</v>
+        <v>30</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1603,29 +1583,27 @@
         <v>44</v>
       </c>
       <c r="G14" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="J14" t="n">
-        <v>27</v>
+        <v>121</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L14" t="n">
+        <v>172</v>
       </c>
       <c r="M14" t="n">
-        <v>172</v>
+        <v>28</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -1697,23 +1675,21 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="J15" t="n">
-        <v>21</v>
+        <v>155</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>:</t>
-        </is>
+      <c r="L15" t="n">
+        <v>198</v>
       </c>
       <c r="M15" t="n">
-        <v>198</v>
+        <v>28</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -15478,7 +15454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16082,126 +16058,6 @@
         </is>
       </c>
       <c r="D48" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>TODO-auto</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>[TBD] tabulka (re-extrakce): chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
         <is>
           <t>TODO-auto</t>
         </is>
@@ -48372,7 +48228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -49295,208 +49151,8 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>TJ Motor České Budějovice</t>
-        </is>
-      </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>TJ Poldi SONP Kladno</t>
-        </is>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>TJ Dukla Jihlava</t>
-        </is>
-      </c>
-      <c r="D48" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>TJ CHZ Litvínov</t>
-        </is>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>TJ Dukla Trenčín</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>TJ Tesla Pardubice</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>TJ Sparta ČKD Praha</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>TJ VSŽ Košice</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>TJ Gottwaldov</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>tabulka (re-extrakce)</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>TJ Škoda Plzeň</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>chybí obdržené branky (GA) — doplnit ze zdroje</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F55"/>
+  <autoFilter ref="A1:F45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>